<commit_message>
Fix Excel save for Streamlit cloud
</commit_message>
<xml_diff>
--- a/test6.xlsx
+++ b/test6.xlsx
@@ -596,7 +596,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O30"/>
+  <dimension ref="A1:Q26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -607,70 +607,80 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
+          <t>Measured Date</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
           <t>Machine</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Part Type</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Chamber</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Piece ID</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Part In/Out</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Batch Cleaning</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Hole</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Feature</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Value</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>Nominal</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>LSL</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>USL</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>Image Path</t>
         </is>
@@ -684,52 +694,57 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
+          <t>2025-11-03</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
           <t>SA01</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="D2" t="inlineStr">
         <is>
           <t>Mixing Block</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="E2" t="inlineStr">
         <is>
           <t>B</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="F2" t="inlineStr">
         <is>
           <t>301390-1923-M840</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="G2" t="inlineStr">
         <is>
           <t>IN</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="I2" t="inlineStr">
         <is>
           <t>H1</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
+      <c r="J2" t="inlineStr">
         <is>
           <t>Inner</t>
         </is>
       </c>
-      <c r="I2" t="n">
+      <c r="K2" t="n">
         <v>4.03</v>
       </c>
-      <c r="J2" t="n">
+      <c r="L2" t="n">
         <v>4</v>
       </c>
-      <c r="K2" t="n">
+      <c r="M2" t="n">
         <v>3.5</v>
       </c>
-      <c r="L2" t="n">
+      <c r="N2" t="n">
         <v>4.5</v>
       </c>
-      <c r="M2" t="inlineStr">
+      <c r="O2" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -743,52 +758,57 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
+          <t>2025-11-03</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
           <t>SA01</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="D3" t="inlineStr">
         <is>
           <t>Mixing Block</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="E3" t="inlineStr">
         <is>
           <t>B</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="F3" t="inlineStr">
         <is>
           <t>301390-1923-M840</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="G3" t="inlineStr">
         <is>
           <t>IN</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
+      <c r="I3" t="inlineStr">
         <is>
           <t>H1</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr">
+      <c r="J3" t="inlineStr">
         <is>
           <t>Outer</t>
         </is>
       </c>
-      <c r="I3" t="n">
+      <c r="K3" t="n">
         <v>9.050000000000001</v>
       </c>
-      <c r="J3" t="n">
+      <c r="L3" t="n">
         <v>9</v>
       </c>
-      <c r="K3" t="n">
+      <c r="M3" t="n">
         <v>8.5</v>
       </c>
-      <c r="L3" t="n">
+      <c r="N3" t="n">
         <v>9.5</v>
       </c>
-      <c r="M3" t="inlineStr">
+      <c r="O3" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -802,52 +822,57 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
+          <t>2025-11-03</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
           <t>SA01</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="D4" t="inlineStr">
         <is>
           <t>Mixing Block</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="E4" t="inlineStr">
         <is>
           <t>B</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
+      <c r="F4" t="inlineStr">
         <is>
           <t>301390-1923-M840</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
+      <c r="G4" t="inlineStr">
         <is>
           <t>IN</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr">
+      <c r="I4" t="inlineStr">
         <is>
           <t>H2</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr">
+      <c r="J4" t="inlineStr">
         <is>
           <t>Inner</t>
         </is>
       </c>
-      <c r="I4" t="n">
+      <c r="K4" t="n">
         <v>4.04</v>
       </c>
-      <c r="J4" t="n">
+      <c r="L4" t="n">
         <v>4</v>
       </c>
-      <c r="K4" t="n">
+      <c r="M4" t="n">
         <v>3.5</v>
       </c>
-      <c r="L4" t="n">
+      <c r="N4" t="n">
         <v>4.5</v>
       </c>
-      <c r="M4" t="inlineStr">
+      <c r="O4" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -861,52 +886,57 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
+          <t>2025-11-03</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
           <t>SA01</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="D5" t="inlineStr">
         <is>
           <t>Mixing Block</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="E5" t="inlineStr">
         <is>
           <t>B</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr">
+      <c r="F5" t="inlineStr">
         <is>
           <t>301390-1923-M840</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr">
+      <c r="G5" t="inlineStr">
         <is>
           <t>IN</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr">
+      <c r="I5" t="inlineStr">
         <is>
           <t>H2</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr">
+      <c r="J5" t="inlineStr">
         <is>
           <t>Outer</t>
         </is>
       </c>
-      <c r="I5" t="n">
+      <c r="K5" t="n">
         <v>9.050000000000001</v>
       </c>
-      <c r="J5" t="n">
+      <c r="L5" t="n">
         <v>9</v>
       </c>
-      <c r="K5" t="n">
+      <c r="M5" t="n">
         <v>8.5</v>
       </c>
-      <c r="L5" t="n">
+      <c r="N5" t="n">
         <v>9.5</v>
       </c>
-      <c r="M5" t="inlineStr">
+      <c r="O5" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -920,52 +950,57 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
+          <t>2025-11-03</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
           <t>SA01</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="D6" t="inlineStr">
         <is>
           <t>Mixing Block</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
+      <c r="E6" t="inlineStr">
         <is>
           <t>B</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr">
+      <c r="F6" t="inlineStr">
         <is>
           <t>301390-1923-M840</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr">
+      <c r="G6" t="inlineStr">
         <is>
           <t>IN</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr">
+      <c r="I6" t="inlineStr">
         <is>
           <t>H3</t>
         </is>
       </c>
-      <c r="H6" t="inlineStr">
+      <c r="J6" t="inlineStr">
         <is>
           <t>Inner</t>
         </is>
       </c>
-      <c r="I6" t="n">
+      <c r="K6" t="n">
         <v>6.24</v>
       </c>
-      <c r="J6" t="n">
+      <c r="L6" t="n">
         <v>6.4</v>
       </c>
-      <c r="K6" t="n">
+      <c r="M6" t="n">
         <v>5.9</v>
       </c>
-      <c r="L6" t="n">
+      <c r="N6" t="n">
         <v>6.9</v>
       </c>
-      <c r="M6" t="inlineStr">
+      <c r="O6" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -979,52 +1014,57 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
+          <t>2025-11-03</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
           <t>SA01</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="D7" t="inlineStr">
         <is>
           <t>Mixing Block</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
+      <c r="E7" t="inlineStr">
         <is>
           <t>B</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr">
+      <c r="F7" t="inlineStr">
         <is>
           <t>301390-1923-M840</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr">
+      <c r="G7" t="inlineStr">
         <is>
           <t>IN</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr">
+      <c r="I7" t="inlineStr">
         <is>
           <t>H3</t>
         </is>
       </c>
-      <c r="H7" t="inlineStr">
+      <c r="J7" t="inlineStr">
         <is>
           <t>Outer</t>
         </is>
       </c>
-      <c r="I7" t="n">
+      <c r="K7" t="n">
         <v>9.029999999999999</v>
       </c>
-      <c r="J7" t="n">
+      <c r="L7" t="n">
         <v>9.199999999999999</v>
       </c>
-      <c r="K7" t="n">
+      <c r="M7" t="n">
         <v>8.699999999999999</v>
       </c>
-      <c r="L7" t="n">
+      <c r="N7" t="n">
         <v>9.699999999999999</v>
       </c>
-      <c r="M7" t="inlineStr">
+      <c r="O7" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -1038,52 +1078,57 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
+          <t>2025-11-03</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
           <t>SA01</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
+      <c r="D8" t="inlineStr">
         <is>
           <t>Mixing Block</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr">
+      <c r="E8" t="inlineStr">
         <is>
           <t>B</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr">
+      <c r="F8" t="inlineStr">
         <is>
           <t>301390-1923-M840</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr">
+      <c r="G8" t="inlineStr">
         <is>
           <t>IN</t>
         </is>
       </c>
-      <c r="G8" t="inlineStr">
+      <c r="I8" t="inlineStr">
         <is>
           <t>H4</t>
         </is>
       </c>
-      <c r="H8" t="inlineStr">
+      <c r="J8" t="inlineStr">
         <is>
           <t>Inner</t>
         </is>
       </c>
-      <c r="I8" t="n">
+      <c r="K8" t="n">
         <v>9.16</v>
       </c>
-      <c r="J8" t="n">
+      <c r="L8" t="n">
         <v>9.199999999999999</v>
       </c>
-      <c r="K8" t="n">
+      <c r="M8" t="n">
         <v>8.699999999999999</v>
       </c>
-      <c r="L8" t="n">
+      <c r="N8" t="n">
         <v>9.699999999999999</v>
       </c>
-      <c r="M8" t="inlineStr">
+      <c r="O8" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -1097,58 +1142,64 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
+          <t>2025-11-03</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
           <t>SA01</t>
         </is>
       </c>
-      <c r="C9" s="2" t="inlineStr">
+      <c r="D9" s="2" t="inlineStr">
         <is>
           <t>Mixing Block</t>
         </is>
       </c>
-      <c r="D9" s="2" t="inlineStr">
+      <c r="E9" s="2" t="inlineStr">
         <is>
           <t>B</t>
         </is>
       </c>
-      <c r="E9" s="2" t="inlineStr">
+      <c r="F9" s="2" t="inlineStr">
         <is>
           <t>301390-1923-M840</t>
         </is>
       </c>
-      <c r="F9" s="2" t="inlineStr">
+      <c r="G9" s="2" t="inlineStr">
         <is>
           <t>IN</t>
         </is>
       </c>
-      <c r="G9" s="2" t="inlineStr">
+      <c r="H9" s="2" t="n"/>
+      <c r="I9" s="2" t="inlineStr">
         <is>
           <t>H4</t>
         </is>
       </c>
-      <c r="H9" s="2" t="inlineStr">
+      <c r="J9" s="2" t="inlineStr">
         <is>
           <t>Outer</t>
         </is>
       </c>
-      <c r="I9" s="2" t="n">
+      <c r="K9" s="2" t="n">
         <v>12.82</v>
       </c>
-      <c r="J9" s="2" t="n">
+      <c r="L9" s="2" t="n">
         <v>12.8</v>
       </c>
-      <c r="K9" s="2" t="n">
+      <c r="M9" s="2" t="n">
         <v>12.3</v>
       </c>
-      <c r="L9" s="2" t="n">
+      <c r="N9" s="2" t="n">
         <v>13.3</v>
       </c>
-      <c r="M9" s="2" t="inlineStr">
+      <c r="O9" s="2" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
       </c>
-      <c r="N9" s="2" t="n"/>
-      <c r="O9" s="2" t="n"/>
+      <c r="P9" s="2" t="n"/>
+      <c r="Q9" s="2" t="n"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1158,59 +1209,62 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
+          <t>2025-11-06</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
           <t>SA03</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
+      <c r="D10" t="inlineStr">
         <is>
           <t>Mixing Block</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr">
+      <c r="E10" t="inlineStr">
         <is>
           <t>D</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr">
+      <c r="F10" t="inlineStr">
         <is>
           <t>301390-3321-M455</t>
         </is>
       </c>
-      <c r="F10" t="inlineStr">
+      <c r="G10" t="inlineStr">
         <is>
           <t>IN</t>
         </is>
       </c>
-      <c r="G10" t="inlineStr">
+      <c r="H10" t="n">
+        <v>3</v>
+      </c>
+      <c r="I10" t="inlineStr">
         <is>
           <t>H1</t>
         </is>
       </c>
-      <c r="H10" t="inlineStr">
+      <c r="J10" t="inlineStr">
         <is>
           <t>Inner</t>
         </is>
       </c>
-      <c r="I10" t="n">
+      <c r="K10" t="n">
         <v>4.13</v>
       </c>
-      <c r="J10" t="n">
+      <c r="L10" t="n">
         <v>4</v>
       </c>
-      <c r="K10" t="n">
+      <c r="M10" t="n">
         <v>3.5</v>
       </c>
-      <c r="L10" t="n">
+      <c r="N10" t="n">
         <v>4.5</v>
       </c>
-      <c r="M10" t="inlineStr">
+      <c r="O10" t="inlineStr">
         <is>
           <t>PASS</t>
-        </is>
-      </c>
-      <c r="N10" t="inlineStr">
-        <is>
-          <t>3rd batch cleaning</t>
         </is>
       </c>
     </row>
@@ -1222,59 +1276,62 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
+          <t>2025-11-06</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
           <t>SA03</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr">
+      <c r="D11" t="inlineStr">
         <is>
           <t>Mixing Block</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr">
+      <c r="E11" t="inlineStr">
         <is>
           <t>D</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr">
+      <c r="F11" t="inlineStr">
         <is>
           <t>301390-3321-M455</t>
         </is>
       </c>
-      <c r="F11" t="inlineStr">
+      <c r="G11" t="inlineStr">
         <is>
           <t>IN</t>
         </is>
       </c>
-      <c r="G11" t="inlineStr">
+      <c r="H11" t="n">
+        <v>3</v>
+      </c>
+      <c r="I11" t="inlineStr">
         <is>
           <t>H1</t>
         </is>
       </c>
-      <c r="H11" t="inlineStr">
+      <c r="J11" t="inlineStr">
         <is>
           <t>Outer</t>
         </is>
       </c>
-      <c r="I11" t="n">
+      <c r="K11" t="n">
         <v>9.01</v>
       </c>
-      <c r="J11" t="n">
+      <c r="L11" t="n">
         <v>9</v>
       </c>
-      <c r="K11" t="n">
+      <c r="M11" t="n">
         <v>8.5</v>
       </c>
-      <c r="L11" t="n">
+      <c r="N11" t="n">
         <v>9.5</v>
       </c>
-      <c r="M11" t="inlineStr">
+      <c r="O11" t="inlineStr">
         <is>
           <t>PASS</t>
-        </is>
-      </c>
-      <c r="N11" t="inlineStr">
-        <is>
-          <t>3rd batch cleaning</t>
         </is>
       </c>
     </row>
@@ -1286,59 +1343,62 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
+          <t>2025-11-06</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
           <t>SA03</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr">
+      <c r="D12" t="inlineStr">
         <is>
           <t>Mixing Block</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr">
+      <c r="E12" t="inlineStr">
         <is>
           <t>D</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr">
+      <c r="F12" t="inlineStr">
         <is>
           <t>301390-3321-M455</t>
         </is>
       </c>
-      <c r="F12" t="inlineStr">
+      <c r="G12" t="inlineStr">
         <is>
           <t>IN</t>
         </is>
       </c>
-      <c r="G12" t="inlineStr">
+      <c r="H12" t="n">
+        <v>3</v>
+      </c>
+      <c r="I12" t="inlineStr">
         <is>
           <t>H2</t>
         </is>
       </c>
-      <c r="H12" t="inlineStr">
+      <c r="J12" t="inlineStr">
         <is>
           <t>Inner</t>
         </is>
       </c>
-      <c r="I12" t="n">
-        <v>4.15</v>
-      </c>
-      <c r="J12" t="n">
+      <c r="K12" t="n">
+        <v>4.04</v>
+      </c>
+      <c r="L12" t="n">
         <v>4</v>
       </c>
-      <c r="K12" t="n">
+      <c r="M12" t="n">
         <v>3.5</v>
       </c>
-      <c r="L12" t="n">
+      <c r="N12" t="n">
         <v>4.5</v>
       </c>
-      <c r="M12" t="inlineStr">
+      <c r="O12" t="inlineStr">
         <is>
           <t>PASS</t>
-        </is>
-      </c>
-      <c r="N12" t="inlineStr">
-        <is>
-          <t>3rd batch cleaning</t>
         </is>
       </c>
     </row>
@@ -1350,59 +1410,62 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
+          <t>2025-11-06</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
           <t>SA03</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr">
+      <c r="D13" t="inlineStr">
         <is>
           <t>Mixing Block</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr">
+      <c r="E13" t="inlineStr">
         <is>
           <t>D</t>
         </is>
       </c>
-      <c r="E13" t="inlineStr">
+      <c r="F13" t="inlineStr">
         <is>
           <t>301390-3321-M455</t>
         </is>
       </c>
-      <c r="F13" t="inlineStr">
+      <c r="G13" t="inlineStr">
         <is>
           <t>IN</t>
         </is>
       </c>
-      <c r="G13" t="inlineStr">
+      <c r="H13" t="n">
+        <v>3</v>
+      </c>
+      <c r="I13" t="inlineStr">
         <is>
           <t>H2</t>
         </is>
       </c>
-      <c r="H13" t="inlineStr">
+      <c r="J13" t="inlineStr">
         <is>
           <t>Outer</t>
         </is>
       </c>
-      <c r="I13" t="n">
+      <c r="K13" t="n">
         <v>9.140000000000001</v>
       </c>
-      <c r="J13" t="n">
+      <c r="L13" t="n">
         <v>9</v>
       </c>
-      <c r="K13" t="n">
+      <c r="M13" t="n">
         <v>8.5</v>
       </c>
-      <c r="L13" t="n">
+      <c r="N13" t="n">
         <v>9.5</v>
       </c>
-      <c r="M13" t="inlineStr">
+      <c r="O13" t="inlineStr">
         <is>
           <t>PASS</t>
-        </is>
-      </c>
-      <c r="N13" t="inlineStr">
-        <is>
-          <t>3rd batch cleaning</t>
         </is>
       </c>
     </row>
@@ -1414,59 +1477,62 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
+          <t>2025-11-06</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
           <t>SA03</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr">
+      <c r="D14" t="inlineStr">
         <is>
           <t>Mixing Block</t>
         </is>
       </c>
-      <c r="D14" t="inlineStr">
+      <c r="E14" t="inlineStr">
         <is>
           <t>D</t>
         </is>
       </c>
-      <c r="E14" t="inlineStr">
+      <c r="F14" t="inlineStr">
         <is>
           <t>301390-3321-M455</t>
         </is>
       </c>
-      <c r="F14" t="inlineStr">
+      <c r="G14" t="inlineStr">
         <is>
           <t>IN</t>
         </is>
       </c>
-      <c r="G14" t="inlineStr">
+      <c r="H14" t="n">
+        <v>3</v>
+      </c>
+      <c r="I14" t="inlineStr">
         <is>
           <t>H3</t>
         </is>
       </c>
-      <c r="H14" t="inlineStr">
+      <c r="J14" t="inlineStr">
         <is>
           <t>Inner</t>
         </is>
       </c>
-      <c r="I14" t="n">
+      <c r="K14" t="n">
         <v>6.87</v>
       </c>
-      <c r="J14" t="n">
+      <c r="L14" t="n">
         <v>6.4</v>
       </c>
-      <c r="K14" t="n">
+      <c r="M14" t="n">
         <v>5.9</v>
       </c>
-      <c r="L14" t="n">
+      <c r="N14" t="n">
         <v>6.9</v>
       </c>
-      <c r="M14" t="inlineStr">
+      <c r="O14" t="inlineStr">
         <is>
           <t>PASS</t>
-        </is>
-      </c>
-      <c r="N14" t="inlineStr">
-        <is>
-          <t>3rd batch cleaning</t>
         </is>
       </c>
     </row>
@@ -1478,59 +1544,62 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
+          <t>2025-11-06</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
           <t>SA03</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr">
+      <c r="D15" t="inlineStr">
         <is>
           <t>Mixing Block</t>
         </is>
       </c>
-      <c r="D15" t="inlineStr">
+      <c r="E15" t="inlineStr">
         <is>
           <t>D</t>
         </is>
       </c>
-      <c r="E15" t="inlineStr">
+      <c r="F15" t="inlineStr">
         <is>
           <t>301390-3321-M455</t>
         </is>
       </c>
-      <c r="F15" t="inlineStr">
+      <c r="G15" t="inlineStr">
         <is>
           <t>IN</t>
         </is>
       </c>
-      <c r="G15" t="inlineStr">
+      <c r="H15" t="n">
+        <v>3</v>
+      </c>
+      <c r="I15" t="inlineStr">
         <is>
           <t>H3</t>
         </is>
       </c>
-      <c r="H15" t="inlineStr">
+      <c r="J15" t="inlineStr">
         <is>
           <t>Outer</t>
         </is>
       </c>
-      <c r="I15" t="n">
+      <c r="K15" t="n">
         <v>8.99</v>
       </c>
-      <c r="J15" t="n">
+      <c r="L15" t="n">
         <v>9.199999999999999</v>
       </c>
-      <c r="K15" t="n">
+      <c r="M15" t="n">
         <v>8.699999999999999</v>
       </c>
-      <c r="L15" t="n">
+      <c r="N15" t="n">
         <v>9.699999999999999</v>
       </c>
-      <c r="M15" t="inlineStr">
+      <c r="O15" t="inlineStr">
         <is>
           <t>PASS</t>
-        </is>
-      </c>
-      <c r="N15" t="inlineStr">
-        <is>
-          <t>3rd batch cleaning</t>
         </is>
       </c>
     </row>
@@ -1542,59 +1611,62 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
+          <t>2025-11-06</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
           <t>SA03</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr">
+      <c r="D16" t="inlineStr">
         <is>
           <t>Mixing Block</t>
         </is>
       </c>
-      <c r="D16" t="inlineStr">
+      <c r="E16" t="inlineStr">
         <is>
           <t>D</t>
         </is>
       </c>
-      <c r="E16" t="inlineStr">
+      <c r="F16" t="inlineStr">
         <is>
           <t>301390-3321-M455</t>
         </is>
       </c>
-      <c r="F16" t="inlineStr">
+      <c r="G16" t="inlineStr">
         <is>
           <t>IN</t>
         </is>
       </c>
-      <c r="G16" t="inlineStr">
+      <c r="H16" t="n">
+        <v>3</v>
+      </c>
+      <c r="I16" t="inlineStr">
         <is>
           <t>H4</t>
         </is>
       </c>
-      <c r="H16" t="inlineStr">
+      <c r="J16" t="inlineStr">
         <is>
           <t>Inner</t>
         </is>
       </c>
-      <c r="I16" t="n">
+      <c r="K16" t="n">
         <v>9.619999999999999</v>
       </c>
-      <c r="J16" t="n">
+      <c r="L16" t="n">
         <v>9.199999999999999</v>
       </c>
-      <c r="K16" t="n">
+      <c r="M16" t="n">
         <v>8.699999999999999</v>
       </c>
-      <c r="L16" t="n">
+      <c r="N16" t="n">
         <v>9.699999999999999</v>
       </c>
-      <c r="M16" t="inlineStr">
+      <c r="O16" t="inlineStr">
         <is>
           <t>PASS</t>
-        </is>
-      </c>
-      <c r="N16" t="inlineStr">
-        <is>
-          <t>3rd batch cleaning</t>
         </is>
       </c>
     </row>
@@ -1606,62 +1678,66 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
+          <t>2025-11-06</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
           <t>SA03</t>
         </is>
       </c>
-      <c r="C17" s="2" t="inlineStr">
+      <c r="D17" s="2" t="inlineStr">
         <is>
           <t>Mixing Block</t>
         </is>
       </c>
-      <c r="D17" s="2" t="inlineStr">
+      <c r="E17" s="2" t="inlineStr">
         <is>
           <t>D</t>
         </is>
       </c>
-      <c r="E17" s="2" t="inlineStr">
+      <c r="F17" s="2" t="inlineStr">
         <is>
           <t>301390-3321-M455</t>
         </is>
       </c>
-      <c r="F17" s="2" t="inlineStr">
+      <c r="G17" s="2" t="inlineStr">
         <is>
           <t>IN</t>
         </is>
       </c>
-      <c r="G17" s="2" t="inlineStr">
+      <c r="H17" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="I17" s="2" t="inlineStr">
         <is>
           <t>H4</t>
         </is>
       </c>
-      <c r="H17" s="2" t="inlineStr">
+      <c r="J17" s="2" t="inlineStr">
         <is>
           <t>Outer</t>
         </is>
       </c>
-      <c r="I17" s="2" t="n">
+      <c r="K17" s="2" t="n">
         <v>12.62</v>
       </c>
-      <c r="J17" s="2" t="n">
+      <c r="L17" s="2" t="n">
         <v>12.8</v>
       </c>
-      <c r="K17" s="2" t="n">
+      <c r="M17" s="2" t="n">
         <v>12.3</v>
       </c>
-      <c r="L17" s="2" t="n">
+      <c r="N17" s="2" t="n">
         <v>13.3</v>
       </c>
-      <c r="M17" s="2" t="inlineStr">
+      <c r="O17" s="2" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
       </c>
-      <c r="N17" s="2" t="inlineStr">
-        <is>
-          <t>3rd batch cleaning</t>
-        </is>
-      </c>
-      <c r="O17" s="2" t="n"/>
+      <c r="P17" s="2" t="n"/>
+      <c r="Q17" s="2" t="n"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1671,59 +1747,62 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
+          <t>2025-11-06</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
           <t>SA03</t>
         </is>
       </c>
-      <c r="C18" t="inlineStr">
+      <c r="D18" t="inlineStr">
         <is>
           <t>Mixing Block</t>
         </is>
       </c>
-      <c r="D18" t="inlineStr">
+      <c r="E18" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="E18" t="inlineStr">
+      <c r="F18" t="inlineStr">
         <is>
           <t>301390-1322-M593</t>
         </is>
       </c>
-      <c r="F18" t="inlineStr">
+      <c r="G18" t="inlineStr">
         <is>
           <t>IN</t>
         </is>
       </c>
-      <c r="G18" t="inlineStr">
+      <c r="H18" t="n">
+        <v>3</v>
+      </c>
+      <c r="I18" t="inlineStr">
         <is>
           <t>H1</t>
         </is>
       </c>
-      <c r="H18" t="inlineStr">
+      <c r="J18" t="inlineStr">
         <is>
           <t>Inner</t>
         </is>
       </c>
-      <c r="I18" t="n">
+      <c r="K18" t="n">
         <v>4.06</v>
       </c>
-      <c r="J18" t="n">
+      <c r="L18" t="n">
         <v>4</v>
       </c>
-      <c r="K18" t="n">
+      <c r="M18" t="n">
         <v>3.5</v>
       </c>
-      <c r="L18" t="n">
+      <c r="N18" t="n">
         <v>4.5</v>
       </c>
-      <c r="M18" t="inlineStr">
+      <c r="O18" t="inlineStr">
         <is>
           <t>PASS</t>
-        </is>
-      </c>
-      <c r="N18" t="inlineStr">
-        <is>
-          <t>3rd batch cleaning</t>
         </is>
       </c>
     </row>
@@ -1735,59 +1814,62 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
+          <t>2025-11-06</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
           <t>SA03</t>
         </is>
       </c>
-      <c r="C19" t="inlineStr">
+      <c r="D19" t="inlineStr">
         <is>
           <t>Mixing Block</t>
         </is>
       </c>
-      <c r="D19" t="inlineStr">
+      <c r="E19" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="E19" t="inlineStr">
+      <c r="F19" t="inlineStr">
         <is>
           <t>301390-1322-M593</t>
         </is>
       </c>
-      <c r="F19" t="inlineStr">
+      <c r="G19" t="inlineStr">
         <is>
           <t>IN</t>
         </is>
       </c>
-      <c r="G19" t="inlineStr">
+      <c r="H19" t="n">
+        <v>3</v>
+      </c>
+      <c r="I19" t="inlineStr">
         <is>
           <t>H1</t>
         </is>
       </c>
-      <c r="H19" t="inlineStr">
+      <c r="J19" t="inlineStr">
         <is>
           <t>Outer</t>
         </is>
       </c>
-      <c r="I19" t="n">
+      <c r="K19" t="n">
         <v>9.07</v>
       </c>
-      <c r="J19" t="n">
+      <c r="L19" t="n">
         <v>9</v>
       </c>
-      <c r="K19" t="n">
+      <c r="M19" t="n">
         <v>8.5</v>
       </c>
-      <c r="L19" t="n">
+      <c r="N19" t="n">
         <v>9.5</v>
       </c>
-      <c r="M19" t="inlineStr">
+      <c r="O19" t="inlineStr">
         <is>
           <t>PASS</t>
-        </is>
-      </c>
-      <c r="N19" t="inlineStr">
-        <is>
-          <t>3rd batch cleaning</t>
         </is>
       </c>
     </row>
@@ -1799,59 +1881,62 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
+          <t>2025-11-06</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
           <t>SA03</t>
         </is>
       </c>
-      <c r="C20" t="inlineStr">
+      <c r="D20" t="inlineStr">
         <is>
           <t>Mixing Block</t>
         </is>
       </c>
-      <c r="D20" t="inlineStr">
+      <c r="E20" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="E20" t="inlineStr">
+      <c r="F20" t="inlineStr">
         <is>
           <t>301390-1322-M593</t>
         </is>
       </c>
-      <c r="F20" t="inlineStr">
+      <c r="G20" t="inlineStr">
         <is>
           <t>IN</t>
         </is>
       </c>
-      <c r="G20" t="inlineStr">
+      <c r="H20" t="n">
+        <v>3</v>
+      </c>
+      <c r="I20" t="inlineStr">
         <is>
           <t>H2</t>
         </is>
       </c>
-      <c r="H20" t="inlineStr">
+      <c r="J20" t="inlineStr">
         <is>
           <t>Inner</t>
         </is>
       </c>
-      <c r="I20" t="n">
+      <c r="K20" t="n">
         <v>4.03</v>
       </c>
-      <c r="J20" t="n">
+      <c r="L20" t="n">
         <v>4</v>
       </c>
-      <c r="K20" t="n">
+      <c r="M20" t="n">
         <v>3.5</v>
       </c>
-      <c r="L20" t="n">
+      <c r="N20" t="n">
         <v>4.5</v>
       </c>
-      <c r="M20" t="inlineStr">
+      <c r="O20" t="inlineStr">
         <is>
           <t>PASS</t>
-        </is>
-      </c>
-      <c r="N20" t="inlineStr">
-        <is>
-          <t>3rd batch cleaning</t>
         </is>
       </c>
     </row>
@@ -1863,59 +1948,62 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
+          <t>2025-11-06</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
           <t>SA03</t>
         </is>
       </c>
-      <c r="C21" t="inlineStr">
+      <c r="D21" t="inlineStr">
         <is>
           <t>Mixing Block</t>
         </is>
       </c>
-      <c r="D21" t="inlineStr">
+      <c r="E21" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="E21" t="inlineStr">
+      <c r="F21" t="inlineStr">
         <is>
           <t>301390-1322-M593</t>
         </is>
       </c>
-      <c r="F21" t="inlineStr">
+      <c r="G21" t="inlineStr">
         <is>
           <t>IN</t>
         </is>
       </c>
-      <c r="G21" t="inlineStr">
+      <c r="H21" t="n">
+        <v>3</v>
+      </c>
+      <c r="I21" t="inlineStr">
         <is>
           <t>H2</t>
         </is>
       </c>
-      <c r="H21" t="inlineStr">
+      <c r="J21" t="inlineStr">
         <is>
           <t>Outer</t>
         </is>
       </c>
-      <c r="I21" t="n">
+      <c r="K21" t="n">
         <v>9.06</v>
       </c>
-      <c r="J21" t="n">
+      <c r="L21" t="n">
         <v>9</v>
       </c>
-      <c r="K21" t="n">
+      <c r="M21" t="n">
         <v>8.5</v>
       </c>
-      <c r="L21" t="n">
+      <c r="N21" t="n">
         <v>9.5</v>
       </c>
-      <c r="M21" t="inlineStr">
+      <c r="O21" t="inlineStr">
         <is>
           <t>PASS</t>
-        </is>
-      </c>
-      <c r="N21" t="inlineStr">
-        <is>
-          <t>3rd batch cleaning</t>
         </is>
       </c>
     </row>
@@ -1927,59 +2015,62 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
+          <t>2025-11-06</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
           <t>SA03</t>
         </is>
       </c>
-      <c r="C22" t="inlineStr">
+      <c r="D22" t="inlineStr">
         <is>
           <t>Mixing Block</t>
         </is>
       </c>
-      <c r="D22" t="inlineStr">
+      <c r="E22" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="E22" t="inlineStr">
+      <c r="F22" t="inlineStr">
         <is>
           <t>301390-1322-M593</t>
         </is>
       </c>
-      <c r="F22" t="inlineStr">
+      <c r="G22" t="inlineStr">
         <is>
           <t>IN</t>
         </is>
       </c>
-      <c r="G22" t="inlineStr">
+      <c r="H22" t="n">
+        <v>3</v>
+      </c>
+      <c r="I22" t="inlineStr">
         <is>
           <t>H3</t>
         </is>
       </c>
-      <c r="H22" t="inlineStr">
+      <c r="J22" t="inlineStr">
         <is>
           <t>Inner</t>
         </is>
       </c>
-      <c r="I22" t="n">
+      <c r="K22" t="n">
         <v>6.43</v>
       </c>
-      <c r="J22" t="n">
+      <c r="L22" t="n">
         <v>6.4</v>
       </c>
-      <c r="K22" t="n">
+      <c r="M22" t="n">
         <v>5.9</v>
       </c>
-      <c r="L22" t="n">
+      <c r="N22" t="n">
         <v>6.9</v>
       </c>
-      <c r="M22" t="inlineStr">
+      <c r="O22" t="inlineStr">
         <is>
           <t>PASS</t>
-        </is>
-      </c>
-      <c r="N22" t="inlineStr">
-        <is>
-          <t>3rd batch cleaning</t>
         </is>
       </c>
     </row>
@@ -1991,59 +2082,62 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
+          <t>2025-11-06</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
           <t>SA03</t>
         </is>
       </c>
-      <c r="C23" t="inlineStr">
+      <c r="D23" t="inlineStr">
         <is>
           <t>Mixing Block</t>
         </is>
       </c>
-      <c r="D23" t="inlineStr">
+      <c r="E23" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="E23" t="inlineStr">
+      <c r="F23" t="inlineStr">
         <is>
           <t>301390-1322-M593</t>
         </is>
       </c>
-      <c r="F23" t="inlineStr">
+      <c r="G23" t="inlineStr">
         <is>
           <t>IN</t>
         </is>
       </c>
-      <c r="G23" t="inlineStr">
+      <c r="H23" t="n">
+        <v>3</v>
+      </c>
+      <c r="I23" t="inlineStr">
         <is>
           <t>H3</t>
         </is>
       </c>
-      <c r="H23" t="inlineStr">
+      <c r="J23" t="inlineStr">
         <is>
           <t>Outer</t>
         </is>
       </c>
-      <c r="I23" t="n">
+      <c r="K23" t="n">
         <v>9.029999999999999</v>
       </c>
-      <c r="J23" t="n">
+      <c r="L23" t="n">
         <v>9.199999999999999</v>
       </c>
-      <c r="K23" t="n">
+      <c r="M23" t="n">
         <v>8.699999999999999</v>
       </c>
-      <c r="L23" t="n">
+      <c r="N23" t="n">
         <v>9.699999999999999</v>
       </c>
-      <c r="M23" t="inlineStr">
+      <c r="O23" t="inlineStr">
         <is>
           <t>PASS</t>
-        </is>
-      </c>
-      <c r="N23" t="inlineStr">
-        <is>
-          <t>3rd batch cleaning</t>
         </is>
       </c>
     </row>
@@ -2055,59 +2149,62 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
+          <t>2025-11-06</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
           <t>SA03</t>
         </is>
       </c>
-      <c r="C24" t="inlineStr">
+      <c r="D24" t="inlineStr">
         <is>
           <t>Mixing Block</t>
         </is>
       </c>
-      <c r="D24" t="inlineStr">
+      <c r="E24" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="E24" t="inlineStr">
+      <c r="F24" t="inlineStr">
         <is>
           <t>301390-1322-M593</t>
         </is>
       </c>
-      <c r="F24" t="inlineStr">
+      <c r="G24" t="inlineStr">
         <is>
           <t>IN</t>
         </is>
       </c>
-      <c r="G24" t="inlineStr">
+      <c r="H24" t="n">
+        <v>3</v>
+      </c>
+      <c r="I24" t="inlineStr">
         <is>
           <t>H4</t>
         </is>
       </c>
-      <c r="H24" t="inlineStr">
+      <c r="J24" t="inlineStr">
         <is>
           <t>Inner</t>
         </is>
       </c>
-      <c r="I24" t="n">
+      <c r="K24" t="n">
         <v>9.66</v>
       </c>
-      <c r="J24" t="n">
+      <c r="L24" t="n">
         <v>9.199999999999999</v>
       </c>
-      <c r="K24" t="n">
+      <c r="M24" t="n">
         <v>8.699999999999999</v>
       </c>
-      <c r="L24" t="n">
+      <c r="N24" t="n">
         <v>9.699999999999999</v>
       </c>
-      <c r="M24" t="inlineStr">
+      <c r="O24" t="inlineStr">
         <is>
           <t>PASS</t>
-        </is>
-      </c>
-      <c r="N24" t="inlineStr">
-        <is>
-          <t>3rd batch cleaning</t>
         </is>
       </c>
     </row>
@@ -2119,367 +2216,133 @@
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
+          <t>2025-11-06</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
           <t>SA03</t>
         </is>
       </c>
-      <c r="C25" s="2" t="inlineStr">
+      <c r="D25" s="2" t="inlineStr">
         <is>
           <t>Mixing Block</t>
         </is>
       </c>
-      <c r="D25" s="2" t="inlineStr">
+      <c r="E25" s="2" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="E25" s="2" t="inlineStr">
+      <c r="F25" s="2" t="inlineStr">
         <is>
           <t>301390-1322-M593</t>
         </is>
       </c>
-      <c r="F25" s="2" t="inlineStr">
+      <c r="G25" s="2" t="inlineStr">
         <is>
           <t>IN</t>
         </is>
       </c>
-      <c r="G25" s="2" t="inlineStr">
+      <c r="H25" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="I25" s="2" t="inlineStr">
         <is>
           <t>H4</t>
         </is>
       </c>
-      <c r="H25" s="2" t="inlineStr">
+      <c r="J25" s="2" t="inlineStr">
         <is>
           <t>Outer</t>
         </is>
       </c>
-      <c r="I25" s="2" t="n">
+      <c r="K25" s="2" t="n">
         <v>12.67</v>
       </c>
-      <c r="J25" s="2" t="n">
+      <c r="L25" s="2" t="n">
         <v>12.8</v>
       </c>
-      <c r="K25" s="2" t="n">
+      <c r="M25" s="2" t="n">
         <v>12.3</v>
       </c>
-      <c r="L25" s="2" t="n">
+      <c r="N25" s="2" t="n">
         <v>13.3</v>
       </c>
-      <c r="M25" s="2" t="inlineStr">
+      <c r="O25" s="2" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
       </c>
-      <c r="N25" s="2" t="inlineStr">
-        <is>
-          <t>3rd batch cleaning</t>
-        </is>
-      </c>
-      <c r="O25" s="2" t="n"/>
+      <c r="P25" s="2" t="n"/>
+      <c r="Q25" s="2" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="3" t="inlineStr">
         <is>
-          <t>2025-11-20 14:10:56</t>
+          <t>2025-11-24 14:44:52</t>
         </is>
       </c>
       <c r="B26" s="3" t="inlineStr">
         <is>
+          <t>2025-11-24</t>
+        </is>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
           <t>SA01</t>
         </is>
       </c>
-      <c r="C26" s="3" t="inlineStr">
+      <c r="D26" s="3" t="inlineStr">
         <is>
           <t>Mixing Block</t>
         </is>
       </c>
-      <c r="D26" s="3" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
       <c r="E26" s="3" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>A</t>
         </is>
       </c>
       <c r="F26" s="3" t="inlineStr">
         <is>
+          <t>301652-1622-0014</t>
+        </is>
+      </c>
+      <c r="G26" s="3" t="inlineStr">
+        <is>
           <t>IN</t>
         </is>
       </c>
-      <c r="G26" s="3" t="inlineStr">
+      <c r="H26" s="3" t="n"/>
+      <c r="I26" s="3" t="inlineStr">
         <is>
           <t>H1</t>
         </is>
       </c>
-      <c r="H26" s="3" t="inlineStr">
+      <c r="J26" s="3" t="inlineStr">
         <is>
           <t>Inner</t>
         </is>
       </c>
-      <c r="I26" s="3" t="n">
-        <v>6.34</v>
-      </c>
-      <c r="J26" s="3" t="n">
+      <c r="K26" s="3" t="n">
+        <v>11</v>
+      </c>
+      <c r="L26" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="K26" s="3" t="n">
+      <c r="M26" s="3" t="n">
         <v>3.5</v>
       </c>
-      <c r="L26" s="3" t="n">
+      <c r="N26" s="3" t="n">
         <v>4.5</v>
       </c>
-      <c r="M26" s="3" t="inlineStr">
+      <c r="O26" s="3" t="inlineStr">
         <is>
           <t>FAIL</t>
         </is>
       </c>
-      <c r="N26" s="3" t="n"/>
-      <c r="O26" s="3" t="n"/>
-    </row>
-    <row r="27">
-      <c r="A27" s="3" t="inlineStr">
-        <is>
-          <t>2025-11-21 11:04:35</t>
-        </is>
-      </c>
-      <c r="B27" s="3" t="inlineStr">
-        <is>
-          <t>SA01</t>
-        </is>
-      </c>
-      <c r="C27" s="3" t="inlineStr">
-        <is>
-          <t>Mixing Block</t>
-        </is>
-      </c>
-      <c r="D27" s="3" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="E27" s="3" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="F27" s="3" t="inlineStr">
-        <is>
-          <t>IN</t>
-        </is>
-      </c>
-      <c r="G27" s="3" t="inlineStr">
-        <is>
-          <t>H1</t>
-        </is>
-      </c>
-      <c r="H27" s="3" t="inlineStr">
-        <is>
-          <t>Inner</t>
-        </is>
-      </c>
-      <c r="I27" s="3" t="n">
-        <v>6.34</v>
-      </c>
-      <c r="J27" s="3" t="n">
-        <v>4</v>
-      </c>
-      <c r="K27" s="3" t="n">
-        <v>3.5</v>
-      </c>
-      <c r="L27" s="3" t="n">
-        <v>4.5</v>
-      </c>
-      <c r="M27" s="3" t="inlineStr">
-        <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-      <c r="N27" s="3" t="n"/>
-      <c r="O27" s="3" t="n"/>
-    </row>
-    <row r="28">
-      <c r="A28" s="3" t="inlineStr">
-        <is>
-          <t>2025-11-21 14:16:06</t>
-        </is>
-      </c>
-      <c r="B28" s="3" t="inlineStr">
-        <is>
-          <t>SA01</t>
-        </is>
-      </c>
-      <c r="C28" s="3" t="inlineStr">
-        <is>
-          <t>Mixing Block</t>
-        </is>
-      </c>
-      <c r="D28" s="3" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="E28" s="3" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="F28" s="3" t="inlineStr">
-        <is>
-          <t>IN</t>
-        </is>
-      </c>
-      <c r="G28" s="3" t="inlineStr">
-        <is>
-          <t>H1</t>
-        </is>
-      </c>
-      <c r="H28" s="3" t="inlineStr">
-        <is>
-          <t>Inner</t>
-        </is>
-      </c>
-      <c r="I28" s="3" t="n">
-        <v>111</v>
-      </c>
-      <c r="J28" s="3" t="n">
-        <v>4</v>
-      </c>
-      <c r="K28" s="3" t="n">
-        <v>3.5</v>
-      </c>
-      <c r="L28" s="3" t="n">
-        <v>4.5</v>
-      </c>
-      <c r="M28" s="3" t="inlineStr">
-        <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-      <c r="N28" s="3" t="n"/>
-      <c r="O28" s="3" t="n"/>
-    </row>
-    <row r="29">
-      <c r="A29" s="4" t="inlineStr">
-        <is>
-          <t>2025-11-21 14:27:43</t>
-        </is>
-      </c>
-      <c r="B29" s="4" t="inlineStr">
-        <is>
-          <t>SA01</t>
-        </is>
-      </c>
-      <c r="C29" s="4" t="inlineStr">
-        <is>
-          <t>Mixing Block</t>
-        </is>
-      </c>
-      <c r="D29" s="4" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="E29" s="4" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="F29" s="4" t="inlineStr">
-        <is>
-          <t>IN</t>
-        </is>
-      </c>
-      <c r="G29" s="4" t="inlineStr">
-        <is>
-          <t>H1</t>
-        </is>
-      </c>
-      <c r="H29" s="4" t="inlineStr">
-        <is>
-          <t>Inner</t>
-        </is>
-      </c>
-      <c r="I29" s="4" t="n">
-        <v>111</v>
-      </c>
-      <c r="J29" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="K29" s="4" t="n">
-        <v>3.5</v>
-      </c>
-      <c r="L29" s="4" t="n">
-        <v>4.5</v>
-      </c>
-      <c r="M29" s="4" t="inlineStr">
-        <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-      <c r="N29" s="4" t="n"/>
-      <c r="O29" s="4" t="n"/>
-    </row>
-    <row r="30">
-      <c r="A30" s="3" t="inlineStr">
-        <is>
-          <t>2025-11-21 14:27:43</t>
-        </is>
-      </c>
-      <c r="B30" s="3" t="inlineStr">
-        <is>
-          <t>SA01</t>
-        </is>
-      </c>
-      <c r="C30" s="3" t="inlineStr">
-        <is>
-          <t>Mixing Block</t>
-        </is>
-      </c>
-      <c r="D30" s="3" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="E30" s="3" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="F30" s="3" t="inlineStr">
-        <is>
-          <t>IN</t>
-        </is>
-      </c>
-      <c r="G30" s="3" t="inlineStr">
-        <is>
-          <t>H2</t>
-        </is>
-      </c>
-      <c r="H30" s="3" t="inlineStr">
-        <is>
-          <t>Inner</t>
-        </is>
-      </c>
-      <c r="I30" s="3" t="n">
-        <v>111</v>
-      </c>
-      <c r="J30" s="3" t="n">
-        <v>4</v>
-      </c>
-      <c r="K30" s="3" t="n">
-        <v>3.5</v>
-      </c>
-      <c r="L30" s="3" t="n">
-        <v>4.5</v>
-      </c>
-      <c r="M30" s="3" t="inlineStr">
-        <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-      <c r="N30" s="3" t="n"/>
-      <c r="O30" s="3" t="n"/>
+      <c r="P26" s="3" t="n"/>
+      <c r="Q26" s="3" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2492,7 +2355,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O16"/>
+  <dimension ref="A1:Q16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2503,70 +2366,80 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
+          <t>Measured Date</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
           <t>Machine</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Part Type</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Chamber</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Piece ID</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Part In/Out</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Batch Cleaning</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Hole</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Feature</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Value</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>Nominal</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>LSL</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>USL</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>Image Path</t>
         </is>
@@ -2580,52 +2453,57 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
+          <t>2025-11-03</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
           <t>SA01</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="D2" t="inlineStr">
         <is>
           <t>Gas/Water Block</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="E2" t="inlineStr">
         <is>
           <t>B</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="F2" t="inlineStr">
         <is>
           <t>301652-3322-0025</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="G2" t="inlineStr">
         <is>
           <t>IN</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="I2" t="inlineStr">
         <is>
           <t>H1</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
+      <c r="J2" t="inlineStr">
         <is>
           <t>Inner</t>
         </is>
       </c>
-      <c r="I2" t="n">
+      <c r="K2" t="n">
         <v>5.97</v>
       </c>
-      <c r="J2" t="n">
+      <c r="L2" t="n">
         <v>5.9</v>
       </c>
-      <c r="K2" t="n">
+      <c r="M2" t="n">
         <v>5.5</v>
       </c>
-      <c r="L2" t="n">
+      <c r="N2" t="n">
         <v>6.4</v>
       </c>
-      <c r="M2" t="inlineStr">
+      <c r="O2" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -2639,52 +2517,57 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
+          <t>2025-11-03</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
           <t>SA01</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="D3" t="inlineStr">
         <is>
           <t>Gas/Water Block</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="E3" t="inlineStr">
         <is>
           <t>B</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="F3" t="inlineStr">
         <is>
           <t>301652-3322-0025</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="G3" t="inlineStr">
         <is>
           <t>IN</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
+      <c r="I3" t="inlineStr">
         <is>
           <t>H2</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr">
+      <c r="J3" t="inlineStr">
         <is>
           <t>Inner</t>
         </is>
       </c>
-      <c r="I3" t="n">
+      <c r="K3" t="n">
         <v>6.19</v>
       </c>
-      <c r="J3" t="n">
+      <c r="L3" t="n">
         <v>6.15</v>
       </c>
-      <c r="K3" t="n">
+      <c r="M3" t="n">
         <v>5.65</v>
       </c>
-      <c r="L3" t="n">
+      <c r="N3" t="n">
         <v>6.65</v>
       </c>
-      <c r="M3" t="inlineStr">
+      <c r="O3" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -2698,52 +2581,57 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
+          <t>2025-11-03</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
           <t>SA01</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="D4" t="inlineStr">
         <is>
           <t>Gas/Water Block</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="E4" t="inlineStr">
         <is>
           <t>B</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
+      <c r="F4" t="inlineStr">
         <is>
           <t>301652-3322-0025</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
+      <c r="G4" t="inlineStr">
         <is>
           <t>IN</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr">
+      <c r="I4" t="inlineStr">
         <is>
           <t>H3</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr">
+      <c r="J4" t="inlineStr">
         <is>
           <t>Inner</t>
         </is>
       </c>
-      <c r="I4" t="n">
+      <c r="K4" t="n">
         <v>6</v>
       </c>
-      <c r="J4" t="n">
+      <c r="L4" t="n">
         <v>6</v>
       </c>
-      <c r="K4" t="n">
+      <c r="M4" t="n">
         <v>5.5</v>
       </c>
-      <c r="L4" t="n">
+      <c r="N4" t="n">
         <v>6.5</v>
       </c>
-      <c r="M4" t="inlineStr">
+      <c r="O4" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -2757,52 +2645,57 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
+          <t>2025-11-03</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
           <t>SA01</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="D5" t="inlineStr">
         <is>
           <t>Gas/Water Block</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="E5" t="inlineStr">
         <is>
           <t>B</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr">
+      <c r="F5" t="inlineStr">
         <is>
           <t>301652-3322-0025</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr">
+      <c r="G5" t="inlineStr">
         <is>
           <t>IN</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr">
+      <c r="I5" t="inlineStr">
         <is>
           <t>H4</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr">
+      <c r="J5" t="inlineStr">
         <is>
           <t>Inner</t>
         </is>
       </c>
-      <c r="I5" t="n">
+      <c r="K5" t="n">
         <v>6.4</v>
       </c>
-      <c r="J5" t="n">
+      <c r="L5" t="n">
         <v>6.3</v>
       </c>
-      <c r="K5" t="n">
+      <c r="M5" t="n">
         <v>5.8</v>
       </c>
-      <c r="L5" t="n">
+      <c r="N5" t="n">
         <v>6.8</v>
       </c>
-      <c r="M5" t="inlineStr">
+      <c r="O5" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -2816,58 +2709,64 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
+          <t>2025-11-03</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
           <t>SA01</t>
         </is>
       </c>
-      <c r="C6" s="2" t="inlineStr">
+      <c r="D6" s="2" t="inlineStr">
         <is>
           <t>Gas/Water Block</t>
         </is>
       </c>
-      <c r="D6" s="2" t="inlineStr">
+      <c r="E6" s="2" t="inlineStr">
         <is>
           <t>B</t>
         </is>
       </c>
-      <c r="E6" s="2" t="inlineStr">
+      <c r="F6" s="2" t="inlineStr">
         <is>
           <t>301652-3322-0025</t>
         </is>
       </c>
-      <c r="F6" s="2" t="inlineStr">
+      <c r="G6" s="2" t="inlineStr">
         <is>
           <t>IN</t>
         </is>
       </c>
-      <c r="G6" s="2" t="inlineStr">
+      <c r="H6" s="2" t="n"/>
+      <c r="I6" s="2" t="inlineStr">
         <is>
           <t>H5</t>
         </is>
       </c>
-      <c r="H6" s="2" t="inlineStr">
+      <c r="J6" s="2" t="inlineStr">
         <is>
           <t>Inner</t>
         </is>
       </c>
-      <c r="I6" s="2" t="n">
+      <c r="K6" s="2" t="n">
         <v>6.2</v>
       </c>
-      <c r="J6" s="2" t="n">
+      <c r="L6" s="2" t="n">
         <v>6.1</v>
       </c>
-      <c r="K6" s="2" t="n">
+      <c r="M6" s="2" t="n">
         <v>5.6</v>
       </c>
-      <c r="L6" s="2" t="n">
+      <c r="N6" s="2" t="n">
         <v>6.6</v>
       </c>
-      <c r="M6" s="2" t="inlineStr">
+      <c r="O6" s="2" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
       </c>
-      <c r="N6" s="2" t="n"/>
-      <c r="O6" s="2" t="n"/>
+      <c r="P6" s="2" t="n"/>
+      <c r="Q6" s="2" t="n"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -2877,59 +2776,62 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
+          <t>2025-11-06</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
           <t>SA03</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="D7" t="inlineStr">
         <is>
           <t>Gas/Water Block</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
+      <c r="E7" t="inlineStr">
         <is>
           <t>D</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr">
+      <c r="F7" t="inlineStr">
         <is>
           <t>301652-2323-0003</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr">
+      <c r="G7" t="inlineStr">
         <is>
           <t>IN</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr">
+      <c r="H7" t="n">
+        <v>3</v>
+      </c>
+      <c r="I7" t="inlineStr">
         <is>
           <t>H1</t>
         </is>
       </c>
-      <c r="H7" t="inlineStr">
+      <c r="J7" t="inlineStr">
         <is>
           <t>Inner</t>
         </is>
       </c>
-      <c r="I7" t="n">
+      <c r="K7" t="n">
         <v>6.36</v>
       </c>
-      <c r="J7" t="n">
+      <c r="L7" t="n">
         <v>5.9</v>
       </c>
-      <c r="K7" t="n">
+      <c r="M7" t="n">
         <v>5.5</v>
       </c>
-      <c r="L7" t="n">
+      <c r="N7" t="n">
         <v>6.4</v>
       </c>
-      <c r="M7" t="inlineStr">
+      <c r="O7" t="inlineStr">
         <is>
           <t>PASS</t>
-        </is>
-      </c>
-      <c r="N7" t="inlineStr">
-        <is>
-          <t>3rd batch cleaning</t>
         </is>
       </c>
     </row>
@@ -2941,59 +2843,62 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
+          <t>2025-11-06</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
           <t>SA03</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
+      <c r="D8" t="inlineStr">
         <is>
           <t>Gas/Water Block</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr">
+      <c r="E8" t="inlineStr">
         <is>
           <t>D</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr">
+      <c r="F8" t="inlineStr">
         <is>
           <t>301652-2323-0003</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr">
+      <c r="G8" t="inlineStr">
         <is>
           <t>IN</t>
         </is>
       </c>
-      <c r="G8" t="inlineStr">
+      <c r="H8" t="n">
+        <v>3</v>
+      </c>
+      <c r="I8" t="inlineStr">
         <is>
           <t>H2</t>
         </is>
       </c>
-      <c r="H8" t="inlineStr">
+      <c r="J8" t="inlineStr">
         <is>
           <t>Inner</t>
         </is>
       </c>
-      <c r="I8" t="n">
+      <c r="K8" t="n">
         <v>6.41</v>
       </c>
-      <c r="J8" t="n">
+      <c r="L8" t="n">
         <v>6.15</v>
       </c>
-      <c r="K8" t="n">
+      <c r="M8" t="n">
         <v>5.65</v>
       </c>
-      <c r="L8" t="n">
+      <c r="N8" t="n">
         <v>6.65</v>
       </c>
-      <c r="M8" t="inlineStr">
+      <c r="O8" t="inlineStr">
         <is>
           <t>PASS</t>
-        </is>
-      </c>
-      <c r="N8" t="inlineStr">
-        <is>
-          <t>3rd batch cleaning</t>
         </is>
       </c>
     </row>
@@ -3005,59 +2910,62 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
+          <t>2025-11-06</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
           <t>SA03</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
+      <c r="D9" t="inlineStr">
         <is>
           <t>Gas/Water Block</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr">
+      <c r="E9" t="inlineStr">
         <is>
           <t>D</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr">
+      <c r="F9" t="inlineStr">
         <is>
           <t>301652-2323-0003</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr">
+      <c r="G9" t="inlineStr">
         <is>
           <t>IN</t>
         </is>
       </c>
-      <c r="G9" t="inlineStr">
+      <c r="H9" t="n">
+        <v>3</v>
+      </c>
+      <c r="I9" t="inlineStr">
         <is>
           <t>H3</t>
         </is>
       </c>
-      <c r="H9" t="inlineStr">
+      <c r="J9" t="inlineStr">
         <is>
           <t>Inner</t>
         </is>
       </c>
-      <c r="I9" t="n">
+      <c r="K9" t="n">
         <v>6.35</v>
       </c>
-      <c r="J9" t="n">
+      <c r="L9" t="n">
         <v>6</v>
       </c>
-      <c r="K9" t="n">
+      <c r="M9" t="n">
         <v>5.5</v>
       </c>
-      <c r="L9" t="n">
+      <c r="N9" t="n">
         <v>6.5</v>
       </c>
-      <c r="M9" t="inlineStr">
+      <c r="O9" t="inlineStr">
         <is>
           <t>PASS</t>
-        </is>
-      </c>
-      <c r="N9" t="inlineStr">
-        <is>
-          <t>3rd batch cleaning</t>
         </is>
       </c>
     </row>
@@ -3069,59 +2977,62 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
+          <t>2025-11-06</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
           <t>SA03</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
+      <c r="D10" t="inlineStr">
         <is>
           <t>Gas/Water Block</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr">
+      <c r="E10" t="inlineStr">
         <is>
           <t>D</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr">
+      <c r="F10" t="inlineStr">
         <is>
           <t>301652-2323-0003</t>
         </is>
       </c>
-      <c r="F10" t="inlineStr">
+      <c r="G10" t="inlineStr">
         <is>
           <t>IN</t>
         </is>
       </c>
-      <c r="G10" t="inlineStr">
+      <c r="H10" t="n">
+        <v>3</v>
+      </c>
+      <c r="I10" t="inlineStr">
         <is>
           <t>H4</t>
         </is>
       </c>
-      <c r="H10" t="inlineStr">
+      <c r="J10" t="inlineStr">
         <is>
           <t>Inner</t>
         </is>
       </c>
-      <c r="I10" t="n">
+      <c r="K10" t="n">
         <v>6.37</v>
       </c>
-      <c r="J10" t="n">
+      <c r="L10" t="n">
         <v>6.3</v>
       </c>
-      <c r="K10" t="n">
+      <c r="M10" t="n">
         <v>5.8</v>
       </c>
-      <c r="L10" t="n">
+      <c r="N10" t="n">
         <v>6.8</v>
       </c>
-      <c r="M10" t="inlineStr">
+      <c r="O10" t="inlineStr">
         <is>
           <t>PASS</t>
-        </is>
-      </c>
-      <c r="N10" t="inlineStr">
-        <is>
-          <t>3rd batch cleaning</t>
         </is>
       </c>
     </row>
@@ -3133,62 +3044,66 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
+          <t>2025-11-06</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
           <t>SA03</t>
         </is>
       </c>
-      <c r="C11" s="2" t="inlineStr">
+      <c r="D11" s="2" t="inlineStr">
         <is>
           <t>Gas/Water Block</t>
         </is>
       </c>
-      <c r="D11" s="2" t="inlineStr">
+      <c r="E11" s="2" t="inlineStr">
         <is>
           <t>D</t>
         </is>
       </c>
-      <c r="E11" s="2" t="inlineStr">
+      <c r="F11" s="2" t="inlineStr">
         <is>
           <t>301652-2323-0003</t>
         </is>
       </c>
-      <c r="F11" s="2" t="inlineStr">
+      <c r="G11" s="2" t="inlineStr">
         <is>
           <t>IN</t>
         </is>
       </c>
-      <c r="G11" s="2" t="inlineStr">
+      <c r="H11" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="I11" s="2" t="inlineStr">
         <is>
           <t>H5</t>
         </is>
       </c>
-      <c r="H11" s="2" t="inlineStr">
+      <c r="J11" s="2" t="inlineStr">
         <is>
           <t>Inner</t>
         </is>
       </c>
-      <c r="I11" s="2" t="n">
+      <c r="K11" s="2" t="n">
         <v>6.42</v>
       </c>
-      <c r="J11" s="2" t="n">
+      <c r="L11" s="2" t="n">
         <v>6.1</v>
       </c>
-      <c r="K11" s="2" t="n">
+      <c r="M11" s="2" t="n">
         <v>5.6</v>
       </c>
-      <c r="L11" s="2" t="n">
+      <c r="N11" s="2" t="n">
         <v>6.6</v>
       </c>
-      <c r="M11" s="2" t="inlineStr">
+      <c r="O11" s="2" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
       </c>
-      <c r="N11" s="2" t="inlineStr">
-        <is>
-          <t>3rd batch cleaning</t>
-        </is>
-      </c>
-      <c r="O11" s="2" t="n"/>
+      <c r="P11" s="2" t="n"/>
+      <c r="Q11" s="2" t="n"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -3198,59 +3113,62 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
+          <t>2025-11-06</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
           <t>SA03</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr">
+      <c r="D12" t="inlineStr">
         <is>
           <t>Gas/Water Block</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr">
+      <c r="E12" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr">
+      <c r="F12" t="inlineStr">
         <is>
           <t>301652-1622-0014</t>
         </is>
       </c>
-      <c r="F12" t="inlineStr">
+      <c r="G12" t="inlineStr">
         <is>
           <t>IN</t>
         </is>
       </c>
-      <c r="G12" t="inlineStr">
+      <c r="H12" t="n">
+        <v>1</v>
+      </c>
+      <c r="I12" t="inlineStr">
         <is>
           <t>H1</t>
         </is>
       </c>
-      <c r="H12" t="inlineStr">
+      <c r="J12" t="inlineStr">
         <is>
           <t>Inner</t>
         </is>
       </c>
-      <c r="I12" t="n">
+      <c r="K12" t="n">
         <v>6.34</v>
       </c>
-      <c r="J12" t="n">
+      <c r="L12" t="n">
         <v>5.9</v>
       </c>
-      <c r="K12" t="n">
+      <c r="M12" t="n">
         <v>5.5</v>
       </c>
-      <c r="L12" t="n">
+      <c r="N12" t="n">
         <v>6.4</v>
       </c>
-      <c r="M12" t="inlineStr">
+      <c r="O12" t="inlineStr">
         <is>
           <t>PASS</t>
-        </is>
-      </c>
-      <c r="N12" t="inlineStr">
-        <is>
-          <t>1st batch cleaning (rejected)</t>
         </is>
       </c>
     </row>
@@ -3262,59 +3180,62 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
+          <t>2025-11-06</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
           <t>SA03</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr">
+      <c r="D13" t="inlineStr">
         <is>
           <t>Gas/Water Block</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr">
+      <c r="E13" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="E13" t="inlineStr">
+      <c r="F13" t="inlineStr">
         <is>
           <t>301652-1622-0014</t>
         </is>
       </c>
-      <c r="F13" t="inlineStr">
+      <c r="G13" t="inlineStr">
         <is>
           <t>IN</t>
         </is>
       </c>
-      <c r="G13" t="inlineStr">
+      <c r="H13" t="n">
+        <v>1</v>
+      </c>
+      <c r="I13" t="inlineStr">
         <is>
           <t>H2</t>
         </is>
       </c>
-      <c r="H13" t="inlineStr">
+      <c r="J13" t="inlineStr">
         <is>
           <t>Inner</t>
         </is>
       </c>
-      <c r="I13" t="n">
+      <c r="K13" t="n">
         <v>6.11</v>
       </c>
-      <c r="J13" t="n">
+      <c r="L13" t="n">
         <v>6.15</v>
       </c>
-      <c r="K13" t="n">
+      <c r="M13" t="n">
         <v>5.65</v>
       </c>
-      <c r="L13" t="n">
+      <c r="N13" t="n">
         <v>6.65</v>
       </c>
-      <c r="M13" t="inlineStr">
+      <c r="O13" t="inlineStr">
         <is>
           <t>PASS</t>
-        </is>
-      </c>
-      <c r="N13" t="inlineStr">
-        <is>
-          <t>1st batch cleaning (rejected)</t>
         </is>
       </c>
     </row>
@@ -3326,62 +3247,66 @@
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
+          <t>2025-11-06</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="inlineStr">
+        <is>
           <t>SA03</t>
         </is>
       </c>
-      <c r="C14" s="4" t="inlineStr">
+      <c r="D14" s="4" t="inlineStr">
         <is>
           <t>Gas/Water Block</t>
         </is>
       </c>
-      <c r="D14" s="4" t="inlineStr">
+      <c r="E14" s="4" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="E14" s="4" t="inlineStr">
+      <c r="F14" s="4" t="inlineStr">
         <is>
           <t>301652-1622-0014</t>
         </is>
       </c>
-      <c r="F14" s="4" t="inlineStr">
+      <c r="G14" s="4" t="inlineStr">
         <is>
           <t>IN</t>
         </is>
       </c>
-      <c r="G14" s="4" t="inlineStr">
+      <c r="H14" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="I14" s="4" t="inlineStr">
         <is>
           <t>H3</t>
         </is>
       </c>
-      <c r="H14" s="4" t="inlineStr">
+      <c r="J14" s="4" t="inlineStr">
         <is>
           <t>Inner</t>
         </is>
       </c>
-      <c r="I14" s="4" t="n">
+      <c r="K14" s="4" t="n">
         <v>7.84</v>
       </c>
-      <c r="J14" s="4" t="n">
+      <c r="L14" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="K14" s="4" t="n">
+      <c r="M14" s="4" t="n">
         <v>5.5</v>
       </c>
-      <c r="L14" s="4" t="n">
+      <c r="N14" s="4" t="n">
         <v>6.5</v>
       </c>
-      <c r="M14" s="4" t="inlineStr">
+      <c r="O14" s="4" t="inlineStr">
         <is>
           <t>FAIL</t>
         </is>
       </c>
-      <c r="N14" s="4" t="inlineStr">
-        <is>
-          <t>1st batch cleaning (rejected)</t>
-        </is>
-      </c>
-      <c r="O14" s="4" t="inlineStr">
+      <c r="P14" s="4" t="n"/>
+      <c r="Q14" s="4" t="inlineStr">
         <is>
           <t>uploaded_images\H3_Inner.jpg</t>
         </is>
@@ -3395,59 +3320,62 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
+          <t>2025-11-06</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
           <t>SA03</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr">
+      <c r="D15" t="inlineStr">
         <is>
           <t>Gas/Water Block</t>
         </is>
       </c>
-      <c r="D15" t="inlineStr">
+      <c r="E15" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="E15" t="inlineStr">
+      <c r="F15" t="inlineStr">
         <is>
           <t>301652-1622-0014</t>
         </is>
       </c>
-      <c r="F15" t="inlineStr">
+      <c r="G15" t="inlineStr">
         <is>
           <t>IN</t>
         </is>
       </c>
-      <c r="G15" t="inlineStr">
+      <c r="H15" t="n">
+        <v>1</v>
+      </c>
+      <c r="I15" t="inlineStr">
         <is>
           <t>H4</t>
         </is>
       </c>
-      <c r="H15" t="inlineStr">
+      <c r="J15" t="inlineStr">
         <is>
           <t>Inner</t>
         </is>
       </c>
-      <c r="I15" t="n">
+      <c r="K15" t="n">
         <v>6.02</v>
       </c>
-      <c r="J15" t="n">
+      <c r="L15" t="n">
         <v>6.3</v>
       </c>
-      <c r="K15" t="n">
+      <c r="M15" t="n">
         <v>5.8</v>
       </c>
-      <c r="L15" t="n">
+      <c r="N15" t="n">
         <v>6.8</v>
       </c>
-      <c r="M15" t="inlineStr">
+      <c r="O15" t="inlineStr">
         <is>
           <t>PASS</t>
-        </is>
-      </c>
-      <c r="N15" t="inlineStr">
-        <is>
-          <t>1st batch cleaning (rejected)</t>
         </is>
       </c>
     </row>
@@ -3459,62 +3387,66 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
+          <t>2025-11-06</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
           <t>SA03</t>
         </is>
       </c>
-      <c r="C16" s="2" t="inlineStr">
+      <c r="D16" s="2" t="inlineStr">
         <is>
           <t>Gas/Water Block</t>
         </is>
       </c>
-      <c r="D16" s="2" t="inlineStr">
+      <c r="E16" s="2" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="E16" s="2" t="inlineStr">
+      <c r="F16" s="2" t="inlineStr">
         <is>
           <t>301652-1622-0014</t>
         </is>
       </c>
-      <c r="F16" s="2" t="inlineStr">
+      <c r="G16" s="2" t="inlineStr">
         <is>
           <t>IN</t>
         </is>
       </c>
-      <c r="G16" s="2" t="inlineStr">
+      <c r="H16" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="I16" s="2" t="inlineStr">
         <is>
           <t>H5</t>
         </is>
       </c>
-      <c r="H16" s="2" t="inlineStr">
+      <c r="J16" s="2" t="inlineStr">
         <is>
           <t>Inner</t>
         </is>
       </c>
-      <c r="I16" s="2" t="n">
+      <c r="K16" s="2" t="n">
         <v>6.11</v>
       </c>
-      <c r="J16" s="2" t="n">
+      <c r="L16" s="2" t="n">
         <v>6.1</v>
       </c>
-      <c r="K16" s="2" t="n">
+      <c r="M16" s="2" t="n">
         <v>5.6</v>
       </c>
-      <c r="L16" s="2" t="n">
+      <c r="N16" s="2" t="n">
         <v>6.6</v>
       </c>
-      <c r="M16" s="2" t="inlineStr">
+      <c r="O16" s="2" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
       </c>
-      <c r="N16" s="2" t="inlineStr">
-        <is>
-          <t>1st batch cleaning (rejected)</t>
-        </is>
-      </c>
-      <c r="O16" s="2" t="n"/>
+      <c r="P16" s="2" t="n"/>
+      <c r="Q16" s="2" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3816,16 +3748,16 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>5.9</v>
+        <v>6</v>
       </c>
       <c r="E10" t="n">
         <v>5.5</v>
       </c>
       <c r="F10" t="n">
-        <v>6.4</v>
+        <v>6.5</v>
       </c>
       <c r="G10" t="n">
-        <v>0.4</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="11">
@@ -3845,13 +3777,13 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>6.15</v>
+        <v>6</v>
       </c>
       <c r="E11" t="n">
-        <v>5.65</v>
+        <v>5.5</v>
       </c>
       <c r="F11" t="n">
-        <v>6.65</v>
+        <v>6.5</v>
       </c>
       <c r="G11" t="n">
         <v>0.5</v>
@@ -3903,13 +3835,13 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>6.3</v>
+        <v>6</v>
       </c>
       <c r="E13" t="n">
-        <v>5.8</v>
+        <v>5.5</v>
       </c>
       <c r="F13" t="n">
-        <v>6.8</v>
+        <v>6.5</v>
       </c>
       <c r="G13" t="n">
         <v>0.5</v>
@@ -3932,13 +3864,13 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>6.1</v>
+        <v>6</v>
       </c>
       <c r="E14" t="n">
-        <v>5.6</v>
+        <v>5.5</v>
       </c>
       <c r="F14" t="n">
-        <v>6.6</v>
+        <v>6.5</v>
       </c>
       <c r="G14" t="n">
         <v>0.5</v>

</xml_diff>

<commit_message>
Initial commit / update
</commit_message>
<xml_diff>
--- a/test6.xlsx
+++ b/test6.xlsx
@@ -165,7 +165,7 @@
       <row>0</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="10610850" cy="4848225"/>
+    <ext cx="3886200" cy="4800600"/>
     <pic>
       <nvPicPr>
         <cNvPr id="1" name="Image 1" descr="Picture"/>
@@ -193,7 +193,7 @@
       <row>33</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="10610850" cy="4848225"/>
+    <ext cx="2914650" cy="4562475"/>
     <pic>
       <nvPicPr>
         <cNvPr id="2" name="Image 2" descr="Picture"/>
@@ -226,7 +226,7 @@
       <row>0</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="6143625" cy="3838575"/>
+    <ext cx="7191375" cy="4505325"/>
     <pic>
       <nvPicPr>
         <cNvPr id="1" name="Image 1" descr="Picture"/>
@@ -249,12 +249,12 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>10</col>
+      <col>12</col>
       <colOff>0</colOff>
       <row>0</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="7229475" cy="4238625"/>
+    <ext cx="6667500" cy="4467225"/>
     <pic>
       <nvPicPr>
         <cNvPr id="2" name="Image 2" descr="Picture"/>
@@ -277,7 +277,7 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>22</col>
+      <col>23</col>
       <colOff>0</colOff>
       <row>0</row>
       <rowOff>0</rowOff>
@@ -595,7 +595,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q25"/>
+  <dimension ref="A1:R25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -684,11 +684,16 @@
           <t>Image Path</t>
         </is>
       </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>Image Path.1</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2025-11-19 11:59:16</t>
+          <t>2025-11-26 10:20:45</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -752,7 +757,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2025-11-19 11:59:16</t>
+          <t>2025-11-26 10:20:45</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -816,7 +821,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2025-11-19 11:59:16</t>
+          <t>2025-11-26 10:20:45</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -880,7 +885,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2025-11-19 11:59:16</t>
+          <t>2025-11-26 10:20:45</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -944,7 +949,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2025-11-19 11:59:16</t>
+          <t>2025-11-26 10:20:45</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -1008,7 +1013,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2025-11-19 11:59:16</t>
+          <t>2025-11-26 10:20:45</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -1072,7 +1077,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2025-11-19 11:59:16</t>
+          <t>2025-11-26 10:20:45</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -1136,7 +1141,7 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>2025-11-19 11:59:16</t>
+          <t>2025-11-26 10:20:45</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
@@ -1199,11 +1204,12 @@
       </c>
       <c r="P9" s="2" t="n"/>
       <c r="Q9" s="2" t="n"/>
+      <c r="R9" s="2" t="n"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2025-11-19 12:01:42</t>
+          <t>2025-11-26 10:35:32</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -1270,7 +1276,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2025-11-19 12:01:42</t>
+          <t>2025-11-26 10:35:32</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -1337,7 +1343,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2025-11-19 12:01:42</t>
+          <t>2025-11-26 10:35:32</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -1384,7 +1390,7 @@
         </is>
       </c>
       <c r="K12" t="n">
-        <v>4.04</v>
+        <v>4.15</v>
       </c>
       <c r="L12" t="n">
         <v>4</v>
@@ -1404,7 +1410,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2025-11-19 12:01:42</t>
+          <t>2025-11-26 10:35:32</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1471,7 +1477,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2025-11-19 12:01:42</t>
+          <t>2025-11-26 10:35:32</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -1538,7 +1544,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2025-11-19 12:01:42</t>
+          <t>2025-11-26 10:35:32</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1605,7 +1611,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2025-11-19 12:01:42</t>
+          <t>2025-11-26 10:35:32</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -1672,7 +1678,7 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>2025-11-19 12:01:42</t>
+          <t>2025-11-26 10:35:32</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
@@ -1737,11 +1743,12 @@
       </c>
       <c r="P17" s="2" t="n"/>
       <c r="Q17" s="2" t="n"/>
+      <c r="R17" s="2" t="n"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2025-11-19 12:04:29</t>
+          <t>2025-11-26 10:38:40</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -1808,7 +1815,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2025-11-19 12:04:29</t>
+          <t>2025-11-26 10:38:40</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -1875,7 +1882,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2025-11-19 12:04:29</t>
+          <t>2025-11-26 10:38:40</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -1942,7 +1949,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2025-11-19 12:04:29</t>
+          <t>2025-11-26 10:38:40</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -2002,14 +2009,14 @@
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>PASS</t>
+          <t>Pass</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2025-11-19 12:04:29</t>
+          <t>2025-11-26 10:38:40</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -2076,7 +2083,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2025-11-19 12:04:29</t>
+          <t>2025-11-26 10:38:40</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -2143,7 +2150,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2025-11-19 12:04:29</t>
+          <t>2025-11-26 10:38:40</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -2190,7 +2197,7 @@
         </is>
       </c>
       <c r="K24" t="n">
-        <v>9.66</v>
+        <v>9.5</v>
       </c>
       <c r="L24" t="n">
         <v>9.199999999999999</v>
@@ -2203,14 +2210,14 @@
       </c>
       <c r="O24" t="inlineStr">
         <is>
-          <t>PASS</t>
+          <t>Pass</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>2025-11-19 12:04:29</t>
+          <t>2025-11-26 10:38:40</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
@@ -2257,7 +2264,7 @@
         </is>
       </c>
       <c r="K25" s="2" t="n">
-        <v>12.67</v>
+        <v>12.6</v>
       </c>
       <c r="L25" s="2" t="n">
         <v>12.8</v>
@@ -2270,11 +2277,12 @@
       </c>
       <c r="O25" s="2" t="inlineStr">
         <is>
-          <t>PASS</t>
+          <t>Pass</t>
         </is>
       </c>
       <c r="P25" s="2" t="n"/>
       <c r="Q25" s="2" t="n"/>
+      <c r="R25" s="2" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2380,7 +2388,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2025-11-19 12:00:33</t>
+          <t>2025-11-26 10:34:05</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -2427,24 +2435,24 @@
         <v>5.97</v>
       </c>
       <c r="L2" t="n">
-        <v>5.9</v>
+        <v>6</v>
       </c>
       <c r="M2" t="n">
         <v>5.5</v>
       </c>
       <c r="N2" t="n">
-        <v>6.4</v>
+        <v>6.5</v>
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>PASS</t>
+          <t>Pass</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2025-11-19 12:00:33</t>
+          <t>2025-11-26 10:34:05</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -2491,13 +2499,13 @@
         <v>6.19</v>
       </c>
       <c r="L3" t="n">
-        <v>6.15</v>
+        <v>6</v>
       </c>
       <c r="M3" t="n">
-        <v>5.65</v>
+        <v>5.5</v>
       </c>
       <c r="N3" t="n">
-        <v>6.65</v>
+        <v>6.5</v>
       </c>
       <c r="O3" t="inlineStr">
         <is>
@@ -2508,7 +2516,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2025-11-19 12:00:33</t>
+          <t>2025-11-26 10:34:05</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -2572,7 +2580,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2025-11-19 12:00:33</t>
+          <t>2025-11-26 10:34:05</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -2616,16 +2624,16 @@
         </is>
       </c>
       <c r="K5" t="n">
-        <v>6.4</v>
+        <v>6.41</v>
       </c>
       <c r="L5" t="n">
-        <v>6.3</v>
+        <v>6</v>
       </c>
       <c r="M5" t="n">
-        <v>5.8</v>
+        <v>5.5</v>
       </c>
       <c r="N5" t="n">
-        <v>6.8</v>
+        <v>6.5</v>
       </c>
       <c r="O5" t="inlineStr">
         <is>
@@ -2636,7 +2644,7 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>2025-11-19 12:00:33</t>
+          <t>2025-11-26 10:34:05</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
@@ -2681,16 +2689,16 @@
         </is>
       </c>
       <c r="K6" s="2" t="n">
-        <v>6.2</v>
+        <v>6.4</v>
       </c>
       <c r="L6" s="2" t="n">
-        <v>6.1</v>
+        <v>6</v>
       </c>
       <c r="M6" s="2" t="n">
-        <v>5.6</v>
+        <v>5.5</v>
       </c>
       <c r="N6" s="2" t="n">
-        <v>6.6</v>
+        <v>6.5</v>
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
@@ -2703,7 +2711,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2025-11-19 12:02:53</t>
+          <t>2025-11-26 10:36:57</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -2753,13 +2761,13 @@
         <v>6.36</v>
       </c>
       <c r="L7" t="n">
-        <v>5.9</v>
+        <v>6</v>
       </c>
       <c r="M7" t="n">
         <v>5.5</v>
       </c>
       <c r="N7" t="n">
-        <v>6.4</v>
+        <v>6.5</v>
       </c>
       <c r="O7" t="inlineStr">
         <is>
@@ -2770,7 +2778,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2025-11-19 12:02:53</t>
+          <t>2025-11-26 10:36:57</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -2820,13 +2828,13 @@
         <v>6.41</v>
       </c>
       <c r="L8" t="n">
-        <v>6.15</v>
+        <v>6</v>
       </c>
       <c r="M8" t="n">
-        <v>5.65</v>
+        <v>5.5</v>
       </c>
       <c r="N8" t="n">
-        <v>6.65</v>
+        <v>6.5</v>
       </c>
       <c r="O8" t="inlineStr">
         <is>
@@ -2837,7 +2845,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2025-11-19 12:02:53</t>
+          <t>2025-11-26 10:36:57</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -2904,7 +2912,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2025-11-19 12:02:53</t>
+          <t>2025-11-26 10:36:57</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -2954,13 +2962,13 @@
         <v>6.37</v>
       </c>
       <c r="L10" t="n">
-        <v>6.3</v>
+        <v>6</v>
       </c>
       <c r="M10" t="n">
-        <v>5.8</v>
+        <v>5.5</v>
       </c>
       <c r="N10" t="n">
-        <v>6.8</v>
+        <v>6.5</v>
       </c>
       <c r="O10" t="inlineStr">
         <is>
@@ -2971,7 +2979,7 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>2025-11-19 12:02:53</t>
+          <t>2025-11-26 10:36:57</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
@@ -3021,13 +3029,13 @@
         <v>6.42</v>
       </c>
       <c r="L11" s="2" t="n">
-        <v>6.1</v>
+        <v>6</v>
       </c>
       <c r="M11" s="2" t="n">
-        <v>5.6</v>
+        <v>5.5</v>
       </c>
       <c r="N11" s="2" t="n">
-        <v>6.6</v>
+        <v>6.5</v>
       </c>
       <c r="O11" s="2" t="inlineStr">
         <is>
@@ -3040,7 +3048,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2025-11-19 12:05:54</t>
+          <t>2025-11-26 10:40:18</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -3090,13 +3098,13 @@
         <v>6.34</v>
       </c>
       <c r="L12" t="n">
-        <v>5.9</v>
+        <v>6</v>
       </c>
       <c r="M12" t="n">
         <v>5.5</v>
       </c>
       <c r="N12" t="n">
-        <v>6.4</v>
+        <v>6.5</v>
       </c>
       <c r="O12" t="inlineStr">
         <is>
@@ -3107,7 +3115,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2025-11-19 12:05:54</t>
+          <t>2025-11-26 10:40:18</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -3157,13 +3165,13 @@
         <v>6.11</v>
       </c>
       <c r="L13" t="n">
-        <v>6.15</v>
+        <v>6</v>
       </c>
       <c r="M13" t="n">
-        <v>5.65</v>
+        <v>5.5</v>
       </c>
       <c r="N13" t="n">
-        <v>6.65</v>
+        <v>6.5</v>
       </c>
       <c r="O13" t="inlineStr">
         <is>
@@ -3174,7 +3182,7 @@
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>2025-11-19 12:05:54</t>
+          <t>2025-11-26 10:40:18</t>
         </is>
       </c>
       <c r="B14" s="3" t="inlineStr">
@@ -3234,7 +3242,7 @@
       </c>
       <c r="O14" s="3" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>Fail</t>
         </is>
       </c>
       <c r="P14" s="3" t="n"/>
@@ -3247,7 +3255,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2025-11-19 12:05:54</t>
+          <t>2025-11-26 10:40:18</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -3297,13 +3305,13 @@
         <v>6.02</v>
       </c>
       <c r="L15" t="n">
-        <v>6.3</v>
+        <v>6</v>
       </c>
       <c r="M15" t="n">
-        <v>5.8</v>
+        <v>5.5</v>
       </c>
       <c r="N15" t="n">
-        <v>6.8</v>
+        <v>6.5</v>
       </c>
       <c r="O15" t="inlineStr">
         <is>
@@ -3314,7 +3322,7 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>2025-11-19 12:05:54</t>
+          <t>2025-11-26 10:40:18</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
@@ -3364,13 +3372,13 @@
         <v>6.11</v>
       </c>
       <c r="L16" s="2" t="n">
-        <v>6.1</v>
+        <v>6</v>
       </c>
       <c r="M16" s="2" t="n">
-        <v>5.6</v>
+        <v>5.5</v>
       </c>
       <c r="N16" s="2" t="n">
-        <v>6.6</v>
+        <v>6.5</v>
       </c>
       <c r="O16" s="2" t="inlineStr">
         <is>
@@ -3822,8 +3830,8 @@
   <dimension ref="A1:A1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" ht="381.75" customHeight="1"/>
-    <row r="34" ht="381.75" customHeight="1"/>
+    <row r="1" ht="378" customHeight="1"/>
+    <row r="34" ht="359.25" customHeight="1"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -3839,12 +3847,12 @@
   <dimension ref="A1:A1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="92.14285714285714" customWidth="1" min="1" max="1"/>
-    <col width="108.4285714285714" customWidth="1" min="11" max="11"/>
-    <col width="113" customWidth="1" min="23" max="23"/>
+    <col width="107.8571428571429" customWidth="1" min="1" max="1"/>
+    <col width="100" customWidth="1" min="13" max="13"/>
+    <col width="113" customWidth="1" min="24" max="24"/>
   </cols>
   <sheetData>
-    <row r="1" ht="339.75" customHeight="1"/>
+    <row r="1" ht="354.75" customHeight="1"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>

</xml_diff>

<commit_message>
Update app.py and sa.py with new features and bug fixes
</commit_message>
<xml_diff>
--- a/test6.xlsx
+++ b/test6.xlsx
@@ -595,7 +595,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R25"/>
+  <dimension ref="A1:Q25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -684,11 +684,6 @@
           <t>Image Path</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
-        <is>
-          <t>Image Path.1</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -1204,7 +1199,6 @@
       </c>
       <c r="P9" s="2" t="n"/>
       <c r="Q9" s="2" t="n"/>
-      <c r="R9" s="2" t="n"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1743,7 +1737,6 @@
       </c>
       <c r="P17" s="2" t="n"/>
       <c r="Q17" s="2" t="n"/>
-      <c r="R17" s="2" t="n"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -2282,7 +2275,6 @@
       </c>
       <c r="P25" s="2" t="n"/>
       <c r="Q25" s="2" t="n"/>
-      <c r="R25" s="2" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2445,7 +2437,7 @@
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>Pass</t>
+          <t>PASS</t>
         </is>
       </c>
     </row>

</xml_diff>